<commit_message>
updates map to gmap and better routing
</commit_message>
<xml_diff>
--- a/roster demo.xlsx
+++ b/roster demo.xlsx
@@ -1,12 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\barap\OneDrive\Documents\Shaibya Solutions\POC\transportation app\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD6314B9-831E-4AC1-8D49-80EA7441AF9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -641,65 +661,71 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="hh:mm"/>
-  </numFmts>
-  <fonts count="12">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF222222"/>
       <name val="Arial"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF1155CC"/>
       <name val="Georgia"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF222222"/>
       <name val="Georgia"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF1F1F1F"/>
       <name val="Google Sans"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
@@ -709,7 +735,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -731,8 +757,15 @@
     </fill>
   </fills>
   <borders count="6">
-    <border/>
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
@@ -742,6 +775,7 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -756,14 +790,18 @@
       <bottom style="thin">
         <color rgb="FF74777E"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
+      <top/>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -778,175 +816,151 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="29">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="2" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf borderId="2" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="2" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="2" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="3" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
+    <xf numFmtId="20" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
+    <xf numFmtId="20" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="3" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="3" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="3" fillId="3" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="3" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="3" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="3" fillId="3" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="3" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="20" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="3">
     <dxf>
-      <font/>
       <fill>
-        <patternFill patternType="none"/>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
       </fill>
-      <border/>
     </dxf>
     <dxf>
-      <font/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF8F8FF"/>
+          <bgColor rgb="FFF8F8FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF435E91"/>
           <bgColor rgb="FF435E91"/>
         </patternFill>
       </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8F8FF"/>
-          <bgColor rgb="FFF8F8FF"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <border/>
     </dxf>
   </dxfs>
   <tableStyles count="1">
-    <tableStyle count="3" pivot="0" name="Sheet1-style">
-      <tableStyleElement dxfId="1" type="headerRow"/>
-      <tableStyleElement dxfId="2" type="firstRowStripe"/>
-      <tableStyleElement dxfId="3" type="secondRowStripe"/>
+    <tableStyle name="Sheet1-style" pivot="0" count="3" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+      <tableStyleElement type="headerRow" dxfId="2"/>
+      <tableStyleElement type="firstRowStripe" dxfId="1"/>
+      <tableStyleElement type="secondRowStripe" dxfId="0"/>
     </tableStyle>
   </tableStyles>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="J1:P9" displayName="Table_1" name="Table_1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table_1" displayName="Table_1" ref="J1:P9" headerRowCount="0">
   <tableColumns count="7">
-    <tableColumn name="Column1" id="1"/>
-    <tableColumn name="Column2" id="2"/>
-    <tableColumn name="Column3" id="3"/>
-    <tableColumn name="Column4" id="4"/>
-    <tableColumn name="Column5" id="5"/>
-    <tableColumn name="Column6" id="6"/>
-    <tableColumn name="Column7" id="7"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Column1"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Column2"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Column3"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Column4"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Column5"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Column6"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Column7"/>
   </tableColumns>
-  <tableStyleInfo name="Sheet1-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="Sheet1-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion1">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" headerRowCount="1"/>
@@ -956,7 +970,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -1146,17 +1160,27 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:P103"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="36.28515625" customWidth="1"/>
+    <col min="2" max="2" width="135.42578125" customWidth="1"/>
+    <col min="3" max="3" width="37.42578125" customWidth="1"/>
+    <col min="4" max="4" width="34.140625" customWidth="1"/>
+    <col min="7" max="7" width="22" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1188,27 +1212,27 @@
         <v>9</v>
       </c>
       <c r="L1" s="3">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("TRANSPOSE(UNIQUE(FILTER(C:C, C:C&lt;&gt;""Shift Time"", C:C&lt;&gt;""Escort"", C:C&lt;&gt;"""")))"),0.20833333333333334)</f>
-        <v>0.2083333333</v>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("TRANSPOSE(UNIQUE(FILTER(C:C, C:C&lt;&gt;""Shift Time"", C:C&lt;&gt;""Escort"", C:C&lt;&gt;"""")))"),0.208333333333333)</f>
+        <v>0.20833333333333301</v>
       </c>
       <c r="M1" s="3">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.3333333333333333)</f>
-        <v>0.3333333333</v>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.333333333333333)</f>
+        <v>0.33333333333333298</v>
       </c>
       <c r="N1" s="3">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.4791666666666667)</f>
-        <v>0.4791666667</v>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.479166666666666)</f>
+        <v>0.47916666666666602</v>
       </c>
       <c r="O1" s="3">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.4583333333333333)</f>
-        <v>0.4583333333</v>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.458333333333333)</f>
+        <v>0.45833333333333298</v>
       </c>
       <c r="P1" s="3">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.4166666666666667)</f>
-        <v>0.4166666667</v>
-      </c>
-    </row>
-    <row r="2">
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.416666666666666)</f>
+        <v>0.41666666666666602</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>10</v>
       </c>
@@ -1234,38 +1258,38 @@
         <v>15</v>
       </c>
       <c r="J2" s="7" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("UNIQUE(FILTER(G:G, REGEXMATCH(UPPER(G:G), ""^DRIVER[-=]"")))"),"DRIVER-SURAJ")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("UNIQUE(FILTER(G:G, REGEXMATCH(UPPER(G:G), ""^DRIVER[-=]"")))"),"DRIVER-SURAJ")</f>
         <v>DRIVER-SURAJ</v>
       </c>
       <c r="K2" s="8">
-        <v>6.0</v>
-      </c>
-      <c r="L2" s="9" t="str">
-        <f t="shared" ref="L2:P2" si="1">IF(COUNTIFS($G:$G, $J2, $C:$C, L$1)&gt;0, "✓", "")</f>
+        <v>6</v>
+      </c>
+      <c r="L2" s="8" t="str">
+        <f t="shared" ref="L2:P2" ca="1" si="0">IF(COUNTIFS($G:$G, $J2, $C:$C, L$1)&gt;0, "✓", "")</f>
         <v>✓</v>
       </c>
-      <c r="M2" s="9" t="str">
-        <f t="shared" si="1"/>
+      <c r="M2" s="8" t="str">
+        <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
-      <c r="N2" s="9" t="str">
-        <f t="shared" si="1"/>
-        <v>✓</v>
-      </c>
-      <c r="O2" s="9" t="str">
-        <f t="shared" si="1"/>
+      <c r="N2" s="8" t="str">
+        <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
-      <c r="P2" s="9" t="str">
-        <f t="shared" si="1"/>
+      <c r="O2" s="8" t="str">
+        <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="3">
+      <c r="P2" s="8" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v/>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="9" t="s">
         <v>17</v>
       </c>
       <c r="C3" s="5">
@@ -1287,34 +1311,34 @@
         <v>15</v>
       </c>
       <c r="J3" s="7" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Driver-amol")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Driver-amol")</f>
         <v>Driver-amol</v>
       </c>
       <c r="K3" s="8">
-        <v>4.0</v>
-      </c>
-      <c r="L3" s="9" t="str">
-        <f t="shared" ref="L3:P3" si="2">IF(COUNTIFS($G:$G, $J3, $C:$C, L$1)&gt;0, "✓", "")</f>
+        <v>4</v>
+      </c>
+      <c r="L3" s="8" t="str">
+        <f t="shared" ref="L3:P3" ca="1" si="1">IF(COUNTIFS($G:$G, $J3, $C:$C, L$1)&gt;0, "✓", "")</f>
         <v>✓</v>
       </c>
-      <c r="M3" s="9" t="str">
-        <f t="shared" si="2"/>
+      <c r="M3" s="8" t="str">
+        <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
-      <c r="N3" s="9" t="str">
-        <f t="shared" si="2"/>
+      <c r="N3" s="8" t="str">
+        <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
-      <c r="O3" s="9" t="str">
-        <f t="shared" si="2"/>
+      <c r="O3" s="8" t="str">
+        <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
-      <c r="P3" s="9" t="str">
-        <f t="shared" si="2"/>
+      <c r="P3" s="8" t="str">
+        <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>20</v>
       </c>
@@ -1340,34 +1364,34 @@
         <v>24</v>
       </c>
       <c r="J4" s="7" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Driver-Shreekant")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Driver-Shreekant")</f>
         <v>Driver-Shreekant</v>
       </c>
       <c r="K4" s="8">
-        <v>6.0</v>
-      </c>
-      <c r="L4" s="9" t="str">
-        <f t="shared" ref="L4:P4" si="3">IF(COUNTIFS($G:$G, $J4, $C:$C, L$1)&gt;0, "✓", "")</f>
+        <v>6</v>
+      </c>
+      <c r="L4" s="8" t="str">
+        <f t="shared" ref="L4:P4" ca="1" si="2">IF(COUNTIFS($G:$G, $J4, $C:$C, L$1)&gt;0, "✓", "")</f>
         <v>✓</v>
       </c>
-      <c r="M4" s="9" t="str">
-        <f t="shared" si="3"/>
+      <c r="M4" s="8" t="str">
+        <f t="shared" ca="1" si="2"/>
         <v>✓</v>
       </c>
-      <c r="N4" s="9" t="str">
-        <f t="shared" si="3"/>
-        <v>✓</v>
-      </c>
-      <c r="O4" s="9" t="str">
-        <f t="shared" si="3"/>
+      <c r="N4" s="8" t="str">
+        <f t="shared" ca="1" si="2"/>
         <v/>
       </c>
-      <c r="P4" s="9" t="str">
-        <f t="shared" si="3"/>
+      <c r="O4" s="8" t="str">
+        <f t="shared" ca="1" si="2"/>
         <v/>
       </c>
-    </row>
-    <row r="5">
+      <c r="P4" s="8" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>25</v>
       </c>
@@ -1386,39 +1410,39 @@
       <c r="F5" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="G5" s="11"/>
+      <c r="G5" s="10"/>
       <c r="H5" s="4" t="s">
         <v>24</v>
       </c>
       <c r="J5" s="7" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Driver- Ashish")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Driver- Ashish")</f>
         <v>Driver- Ashish</v>
       </c>
       <c r="K5" s="8">
-        <v>4.0</v>
-      </c>
-      <c r="L5" s="9" t="str">
-        <f t="shared" ref="L5:P5" si="4">IF(COUNTIFS($G:$G, $J5, $C:$C, L$1)&gt;0, "✓", "")</f>
+        <v>4</v>
+      </c>
+      <c r="L5" s="8" t="str">
+        <f t="shared" ref="L5:P5" ca="1" si="3">IF(COUNTIFS($G:$G, $J5, $C:$C, L$1)&gt;0, "✓", "")</f>
         <v>✓</v>
       </c>
-      <c r="M5" s="9" t="str">
-        <f t="shared" si="4"/>
+      <c r="M5" s="8" t="str">
+        <f t="shared" ca="1" si="3"/>
         <v>✓</v>
       </c>
-      <c r="N5" s="9" t="str">
-        <f t="shared" si="4"/>
+      <c r="N5" s="8" t="str">
+        <f t="shared" ca="1" si="3"/>
         <v/>
       </c>
-      <c r="O5" s="9" t="str">
-        <f t="shared" si="4"/>
+      <c r="O5" s="8" t="str">
+        <f t="shared" ca="1" si="3"/>
         <v/>
       </c>
-      <c r="P5" s="9" t="str">
-        <f t="shared" si="4"/>
+      <c r="P5" s="8" t="str">
+        <f t="shared" ca="1" si="3"/>
         <v/>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>29</v>
       </c>
@@ -1432,45 +1456,45 @@
         <v>30</v>
       </c>
       <c r="E6" s="5">
-        <v>0.1909722222222222</v>
+        <v>0.19097222222222221</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="11"/>
+      <c r="G6" s="10"/>
       <c r="H6" s="4" t="s">
         <v>24</v>
       </c>
       <c r="J6" s="7" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"DRIVER- ANIKET")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"DRIVER- ANIKET")</f>
         <v>DRIVER- ANIKET</v>
       </c>
       <c r="K6" s="8">
-        <v>6.0</v>
-      </c>
-      <c r="L6" s="9" t="str">
-        <f t="shared" ref="L6:P6" si="5">IF(COUNTIFS($G:$G, $J6, $C:$C, L$1)&gt;0, "✓", "")</f>
+        <v>6</v>
+      </c>
+      <c r="L6" s="8" t="str">
+        <f t="shared" ref="L6:P6" ca="1" si="4">IF(COUNTIFS($G:$G, $J6, $C:$C, L$1)&gt;0, "✓", "")</f>
         <v>✓</v>
       </c>
-      <c r="M6" s="9" t="str">
-        <f t="shared" si="5"/>
+      <c r="M6" s="8" t="str">
+        <f t="shared" ca="1" si="4"/>
         <v>✓</v>
       </c>
-      <c r="N6" s="9" t="str">
-        <f t="shared" si="5"/>
+      <c r="N6" s="8" t="str">
+        <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-      <c r="O6" s="9" t="str">
-        <f t="shared" si="5"/>
+      <c r="O6" s="8" t="str">
+        <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-      <c r="P6" s="9" t="str">
-        <f t="shared" si="5"/>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="12" t="s">
+      <c r="P6" s="8" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A7" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B7" s="4" t="s">
@@ -1488,133 +1512,133 @@
       <c r="F7" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="11"/>
+      <c r="G7" s="10"/>
       <c r="H7" s="4" t="s">
         <v>24</v>
       </c>
       <c r="J7" s="7" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"DRIVER-OM")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"DRIVER-OM")</f>
         <v>DRIVER-OM</v>
       </c>
       <c r="K7" s="8">
-        <v>6.0</v>
-      </c>
-      <c r="L7" s="9" t="str">
-        <f t="shared" ref="L7:P7" si="6">IF(COUNTIFS($G:$G, $J7, $C:$C, L$1)&gt;0, "✓", "")</f>
+        <v>6</v>
+      </c>
+      <c r="L7" s="8" t="str">
+        <f t="shared" ref="L7:P7" ca="1" si="5">IF(COUNTIFS($G:$G, $J7, $C:$C, L$1)&gt;0, "✓", "")</f>
         <v>✓</v>
       </c>
-      <c r="M7" s="9" t="str">
-        <f t="shared" si="6"/>
+      <c r="M7" s="8" t="str">
+        <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
-      <c r="N7" s="9" t="str">
-        <f t="shared" si="6"/>
+      <c r="N7" s="8" t="str">
+        <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
-      <c r="O7" s="9" t="str">
-        <f t="shared" si="6"/>
+      <c r="O7" s="8" t="str">
+        <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
-      <c r="P7" s="9" t="str">
-        <f t="shared" si="6"/>
+      <c r="P7" s="8" t="str">
+        <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="11"/>
-      <c r="B8" s="11"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="11"/>
-      <c r="H8" s="11"/>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A8" s="10"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
       <c r="J8" s="7" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Driver-GOVINDA")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Driver-GOVINDA")</f>
         <v>Driver-GOVINDA</v>
       </c>
       <c r="K8" s="8">
-        <v>4.0</v>
-      </c>
-      <c r="L8" s="9" t="str">
-        <f t="shared" ref="L8:P8" si="7">IF(COUNTIFS($G:$G, $J8, $C:$C, L$1)&gt;0, "✓", "")</f>
+        <v>4</v>
+      </c>
+      <c r="L8" s="8" t="str">
+        <f t="shared" ref="L8:P8" ca="1" si="6">IF(COUNTIFS($G:$G, $J8, $C:$C, L$1)&gt;0, "✓", "")</f>
         <v>✓</v>
       </c>
-      <c r="M8" s="9" t="str">
-        <f t="shared" si="7"/>
+      <c r="M8" s="8" t="str">
+        <f t="shared" ca="1" si="6"/>
         <v/>
       </c>
-      <c r="N8" s="9" t="str">
-        <f t="shared" si="7"/>
+      <c r="N8" s="8" t="str">
+        <f t="shared" ca="1" si="6"/>
         <v/>
       </c>
-      <c r="O8" s="9" t="str">
-        <f t="shared" si="7"/>
+      <c r="O8" s="8" t="str">
+        <f t="shared" ca="1" si="6"/>
         <v/>
       </c>
-      <c r="P8" s="9" t="str">
-        <f t="shared" si="7"/>
+      <c r="P8" s="8" t="str">
+        <f t="shared" ca="1" si="6"/>
         <v/>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="13" t="s">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A9" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G9" s="13" t="s">
+      <c r="G9" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="H9" s="13" t="s">
+      <c r="H9" s="12" t="s">
         <v>7</v>
       </c>
       <c r="J9" s="7" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Driver=Prashant")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Driver=Prashant")</f>
         <v>Driver=Prashant</v>
       </c>
       <c r="K9" s="8">
-        <v>4.0</v>
-      </c>
-      <c r="L9" s="9" t="str">
-        <f t="shared" ref="L9:P9" si="8">IF(COUNTIFS($G:$G, $J9, $C:$C, L$1)&gt;0, "✓", "")</f>
+        <v>4</v>
+      </c>
+      <c r="L9" s="8" t="str">
+        <f t="shared" ref="L9:P9" ca="1" si="7">IF(COUNTIFS($G:$G, $J9, $C:$C, L$1)&gt;0, "✓", "")</f>
         <v/>
       </c>
-      <c r="M9" s="9" t="str">
-        <f t="shared" si="8"/>
+      <c r="M9" s="8" t="str">
+        <f t="shared" ca="1" si="7"/>
         <v>✓</v>
       </c>
-      <c r="N9" s="9" t="str">
-        <f t="shared" si="8"/>
+      <c r="N9" s="8" t="str">
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
-      <c r="O9" s="9" t="str">
-        <f t="shared" si="8"/>
+      <c r="O9" s="8" t="str">
+        <f t="shared" ca="1" si="7"/>
         <v>✓</v>
       </c>
-      <c r="P9" s="9" t="str">
-        <f t="shared" si="8"/>
+      <c r="P9" s="8" t="str">
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="9" t="s">
         <v>35</v>
       </c>
       <c r="C10" s="5">
@@ -1626,7 +1650,7 @@
       <c r="E10" s="5">
         <v>0.1736111111111111</v>
       </c>
-      <c r="F10" s="14" t="s">
+      <c r="F10" s="13" t="s">
         <v>13</v>
       </c>
       <c r="G10" s="6" t="s">
@@ -1636,11 +1660,11 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B11" s="15" t="s">
+      <c r="B11" s="14" t="s">
         <v>39</v>
       </c>
       <c r="C11" s="5">
@@ -1652,7 +1676,7 @@
       <c r="E11" s="5">
         <v>0.18055555555555555</v>
       </c>
-      <c r="F11" s="14" t="s">
+      <c r="F11" s="13" t="s">
         <v>13</v>
       </c>
       <c r="G11" s="6" t="s">
@@ -1662,9 +1686,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="16"/>
-      <c r="B12" s="17" t="s">
+    <row r="12" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="15"/>
+      <c r="B12" s="16" t="s">
         <v>42</v>
       </c>
       <c r="C12" s="5">
@@ -1674,9 +1698,9 @@
         <v>43</v>
       </c>
       <c r="E12" s="5">
-        <v>0.1840277777777778</v>
-      </c>
-      <c r="F12" s="14" t="s">
+        <v>0.18402777777777779</v>
+      </c>
+      <c r="F12" s="13" t="s">
         <v>13</v>
       </c>
       <c r="G12" s="6" t="s">
@@ -1686,43 +1710,43 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="11"/>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="11"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="13" t="s">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A13" s="10"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="10"/>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A14" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B14" s="13" t="s">
+      <c r="B14" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="C14" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D14" s="13" t="s">
+      <c r="D14" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E14" s="13" t="s">
+      <c r="E14" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F14" s="13" t="s">
+      <c r="F14" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G14" s="13" t="s">
+      <c r="G14" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="H14" s="13" t="s">
+      <c r="H14" s="12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
         <v>45</v>
       </c>
@@ -1732,7 +1756,7 @@
       <c r="C15" s="5">
         <v>0.20833333333333334</v>
       </c>
-      <c r="D15" s="15" t="s">
+      <c r="D15" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E15" s="5">
@@ -1741,14 +1765,14 @@
       <c r="F15" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G15" s="18" t="s">
+      <c r="G15" s="17" t="s">
         <v>48</v>
       </c>
       <c r="H15" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
         <v>49</v>
       </c>
@@ -1767,18 +1791,18 @@
       <c r="F16" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="G16" s="18" t="s">
+      <c r="G16" s="17" t="s">
         <v>52</v>
       </c>
       <c r="H16" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="9" t="s">
         <v>54</v>
       </c>
       <c r="C17" s="5">
@@ -1793,18 +1817,18 @@
       <c r="F17" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="G17" s="18" t="s">
+      <c r="G17" s="17" t="s">
         <v>56</v>
       </c>
       <c r="H17" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="19" t="s">
+    <row r="18" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A18" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="28" t="s">
         <v>58</v>
       </c>
       <c r="C18" s="5">
@@ -1814,17 +1838,17 @@
         <v>59</v>
       </c>
       <c r="E18" s="5">
-        <v>0.1840277777777778</v>
+        <v>0.18402777777777779</v>
       </c>
       <c r="F18" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G18" s="11"/>
+      <c r="G18" s="10"/>
       <c r="H18" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
         <v>60</v>
       </c>
@@ -1838,53 +1862,53 @@
         <v>62</v>
       </c>
       <c r="E19" s="5">
-        <v>0.1909722222222222</v>
+        <v>0.19097222222222221</v>
       </c>
       <c r="F19" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G19" s="11"/>
+      <c r="G19" s="10"/>
       <c r="H19" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="20"/>
-      <c r="B20" s="20"/>
-      <c r="C20" s="20"/>
-      <c r="D20" s="20"/>
-      <c r="E20" s="20"/>
-      <c r="F20" s="20"/>
-      <c r="G20" s="20"/>
-      <c r="H20" s="20"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="13" t="s">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A20" s="19"/>
+      <c r="B20" s="19"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="19"/>
+      <c r="G20" s="19"/>
+      <c r="H20" s="19"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A21" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B21" s="13" t="s">
+      <c r="B21" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C21" s="13" t="s">
+      <c r="C21" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D21" s="13" t="s">
+      <c r="D21" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E21" s="13" t="s">
+      <c r="E21" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F21" s="13" t="s">
+      <c r="F21" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G21" s="13" t="s">
+      <c r="G21" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="H21" s="13" t="s">
+      <c r="H21" s="12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>63</v>
       </c>
@@ -1903,22 +1927,22 @@
       <c r="F22" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G22" s="18" t="s">
+      <c r="G22" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="H22" s="15" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="16"/>
-      <c r="B23" s="15" t="s">
+      <c r="H22" s="14" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A23" s="15"/>
+      <c r="B23" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C23" s="5">
         <v>0.20833333333333334</v>
       </c>
-      <c r="D23" s="17" t="s">
+      <c r="D23" s="16" t="s">
         <v>68</v>
       </c>
       <c r="E23" s="5">
@@ -1927,24 +1951,24 @@
       <c r="F23" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G23" s="18" t="s">
+      <c r="G23" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="H23" s="15" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="24">
+      <c r="H23" s="14" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="B24" s="15" t="s">
+      <c r="B24" s="14" t="s">
         <v>71</v>
       </c>
       <c r="C24" s="5">
         <v>0.20833333333333334</v>
       </c>
-      <c r="D24" s="17" t="s">
+      <c r="D24" s="16" t="s">
         <v>72</v>
       </c>
       <c r="E24" s="5">
@@ -1953,68 +1977,68 @@
       <c r="F24" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G24" s="18" t="s">
+      <c r="G24" s="17" t="s">
         <v>73</v>
       </c>
       <c r="H24" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="11"/>
-      <c r="B25" s="11"/>
-      <c r="C25" s="11"/>
-      <c r="D25" s="11"/>
-      <c r="E25" s="11"/>
-      <c r="F25" s="11"/>
-      <c r="G25" s="11"/>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A25" s="10"/>
+      <c r="B25" s="10"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="10"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="10"/>
       <c r="H25" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="13" t="s">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A26" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B26" s="13" t="s">
+      <c r="B26" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C26" s="13" t="s">
+      <c r="C26" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D26" s="13" t="s">
+      <c r="D26" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E26" s="13" t="s">
+      <c r="E26" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F26" s="13" t="s">
+      <c r="F26" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G26" s="13" t="s">
+      <c r="G26" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="H26" s="13" t="s">
+      <c r="H26" s="12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="B27" s="21" t="s">
+      <c r="B27" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="C27" s="21" t="s">
+      <c r="C27" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="D27" s="15" t="s">
+      <c r="D27" s="14" t="s">
         <v>74</v>
       </c>
       <c r="E27" s="5">
         <v>0.125</v>
       </c>
-      <c r="F27" s="15" t="s">
+      <c r="F27" s="14" t="s">
         <v>13</v>
       </c>
       <c r="G27" s="6" t="s">
@@ -2024,7 +2048,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
         <v>76</v>
       </c>
@@ -2038,9 +2062,9 @@
         <v>78</v>
       </c>
       <c r="E28" s="5">
-        <v>0.1597222222222222</v>
-      </c>
-      <c r="F28" s="15" t="s">
+        <v>0.15972222222222221</v>
+      </c>
+      <c r="F28" s="14" t="s">
         <v>13</v>
       </c>
       <c r="G28" s="6" t="s">
@@ -2050,7 +2074,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>80</v>
       </c>
@@ -2066,7 +2090,7 @@
       <c r="E29" s="5">
         <v>0.1701388888888889</v>
       </c>
-      <c r="F29" s="15" t="s">
+      <c r="F29" s="14" t="s">
         <v>13</v>
       </c>
       <c r="G29" s="6" t="s">
@@ -2076,11 +2100,11 @@
         <v>24</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="B30" s="15" t="s">
+      <c r="B30" s="14" t="s">
         <v>85</v>
       </c>
       <c r="C30" s="5">
@@ -2092,15 +2116,15 @@
       <c r="E30" s="5">
         <v>0.17708333333333334</v>
       </c>
-      <c r="F30" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="G30" s="11"/>
+      <c r="F30" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="G30" s="10"/>
       <c r="H30" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
         <v>87</v>
       </c>
@@ -2114,17 +2138,17 @@
         <v>89</v>
       </c>
       <c r="E31" s="5">
-        <v>0.1840277777777778</v>
-      </c>
-      <c r="F31" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="G31" s="11"/>
+        <v>0.18402777777777779</v>
+      </c>
+      <c r="F31" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="G31" s="10"/>
       <c r="H31" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
         <v>90</v>
       </c>
@@ -2140,55 +2164,55 @@
       <c r="E32" s="5">
         <v>0.1875</v>
       </c>
-      <c r="F32" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="G32" s="11"/>
+      <c r="F32" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="G32" s="10"/>
       <c r="H32" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="11"/>
-      <c r="B33" s="11"/>
-      <c r="C33" s="11"/>
-      <c r="D33" s="11"/>
-      <c r="E33" s="11"/>
-      <c r="F33" s="11"/>
-      <c r="G33" s="11"/>
-      <c r="H33" s="11"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="13" t="s">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A33" s="10"/>
+      <c r="B33" s="10"/>
+      <c r="C33" s="10"/>
+      <c r="D33" s="10"/>
+      <c r="E33" s="10"/>
+      <c r="F33" s="10"/>
+      <c r="G33" s="10"/>
+      <c r="H33" s="10"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A34" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B34" s="13" t="s">
+      <c r="B34" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C34" s="13" t="s">
+      <c r="C34" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D34" s="13" t="s">
+      <c r="D34" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E34" s="13" t="s">
+      <c r="E34" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F34" s="13" t="s">
+      <c r="F34" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G34" s="13" t="s">
+      <c r="G34" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="H34" s="13" t="s">
+      <c r="H34" s="12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="B35" s="15" t="s">
+      <c r="B35" s="14" t="s">
         <v>94</v>
       </c>
       <c r="C35" s="5">
@@ -2198,7 +2222,7 @@
         <v>95</v>
       </c>
       <c r="E35" s="5">
-        <v>0.1527777777777778</v>
+        <v>0.15277777777777779</v>
       </c>
       <c r="F35" s="4" t="s">
         <v>13</v>
@@ -2210,7 +2234,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
         <v>97</v>
       </c>
@@ -2236,7 +2260,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
         <v>101</v>
       </c>
@@ -2262,7 +2286,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
         <v>103</v>
       </c>
@@ -2281,13 +2305,13 @@
       <c r="F38" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G38" s="11"/>
+      <c r="G38" s="10"/>
       <c r="H38" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="16"/>
+    <row r="39" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A39" s="15"/>
       <c r="B39" s="4" t="s">
         <v>104</v>
       </c>
@@ -2303,12 +2327,12 @@
       <c r="F39" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G39" s="11"/>
+      <c r="G39" s="10"/>
       <c r="H39" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
         <v>106</v>
       </c>
@@ -2327,48 +2351,48 @@
       <c r="F40" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="G40" s="11"/>
+      <c r="G40" s="10"/>
       <c r="H40" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="11"/>
-      <c r="B41" s="11"/>
-      <c r="C41" s="11"/>
-      <c r="D41" s="11"/>
-      <c r="E41" s="11"/>
-      <c r="F41" s="11"/>
-      <c r="G41" s="11"/>
-      <c r="H41" s="11"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="13" t="s">
+    <row r="41" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A41" s="10"/>
+      <c r="B41" s="10"/>
+      <c r="C41" s="10"/>
+      <c r="D41" s="10"/>
+      <c r="E41" s="10"/>
+      <c r="F41" s="10"/>
+      <c r="G41" s="10"/>
+      <c r="H41" s="10"/>
+    </row>
+    <row r="42" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A42" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B42" s="13" t="s">
+      <c r="B42" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C42" s="13" t="s">
+      <c r="C42" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D42" s="13" t="s">
+      <c r="D42" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E42" s="13" t="s">
+      <c r="E42" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F42" s="13" t="s">
+      <c r="F42" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G42" s="13" t="s">
+      <c r="G42" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="H42" s="13" t="s">
+      <c r="H42" s="12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A43" s="4" t="s">
         <v>108</v>
       </c>
@@ -2387,14 +2411,14 @@
       <c r="F43" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G43" s="22" t="s">
+      <c r="G43" s="21" t="s">
         <v>111</v>
       </c>
       <c r="H43" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
         <v>112</v>
       </c>
@@ -2413,14 +2437,14 @@
       <c r="F44" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G44" s="22" t="s">
+      <c r="G44" s="21" t="s">
         <v>115</v>
       </c>
       <c r="H44" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A45" s="4" t="s">
         <v>116</v>
       </c>
@@ -2439,15 +2463,15 @@
       <c r="F45" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G45" s="22" t="s">
+      <c r="G45" s="21" t="s">
         <v>119</v>
       </c>
       <c r="H45" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="16"/>
+    <row r="46" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A46" s="15"/>
       <c r="B46" s="4" t="s">
         <v>120</v>
       </c>
@@ -2463,48 +2487,48 @@
       <c r="F46" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G46" s="11"/>
+      <c r="G46" s="10"/>
       <c r="H46" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="20"/>
-      <c r="B47" s="20"/>
-      <c r="C47" s="20"/>
-      <c r="D47" s="20"/>
-      <c r="E47" s="20"/>
-      <c r="F47" s="20"/>
-      <c r="G47" s="20"/>
-      <c r="H47" s="20"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="13" t="s">
+    <row r="47" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A47" s="19"/>
+      <c r="B47" s="19"/>
+      <c r="C47" s="19"/>
+      <c r="D47" s="19"/>
+      <c r="E47" s="19"/>
+      <c r="F47" s="19"/>
+      <c r="G47" s="19"/>
+      <c r="H47" s="19"/>
+    </row>
+    <row r="48" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A48" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B48" s="13" t="s">
+      <c r="B48" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C48" s="13" t="s">
+      <c r="C48" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D48" s="13" t="s">
+      <c r="D48" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E48" s="13" t="s">
+      <c r="E48" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F48" s="13" t="s">
+      <c r="F48" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G48" s="13" t="s">
+      <c r="G48" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="H48" s="13" t="s">
+      <c r="H48" s="12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" spans="1:8" ht="15" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
         <v>122</v>
       </c>
@@ -2512,13 +2536,13 @@
         <v>123</v>
       </c>
       <c r="C49" s="5">
-        <v>0.3333333333333333</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="D49" s="4" t="s">
         <v>124</v>
       </c>
       <c r="E49" s="5">
-        <v>0.2916666666666667</v>
+        <v>0.29166666666666669</v>
       </c>
       <c r="F49" s="4" t="s">
         <v>13</v>
@@ -2530,7 +2554,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" spans="1:8" ht="15" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
         <v>126</v>
       </c>
@@ -2538,13 +2562,13 @@
         <v>127</v>
       </c>
       <c r="C50" s="5">
-        <v>0.3333333333333333</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="D50" s="4" t="s">
         <v>128</v>
       </c>
       <c r="E50" s="5">
-        <v>0.3055555555555556</v>
+        <v>0.30555555555555558</v>
       </c>
       <c r="F50" s="4" t="s">
         <v>13</v>
@@ -2556,121 +2580,121 @@
         <v>15</v>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="11"/>
-      <c r="B51" s="11"/>
-      <c r="C51" s="11"/>
-      <c r="D51" s="11"/>
-      <c r="E51" s="11"/>
-      <c r="F51" s="11"/>
+    <row r="51" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="A51" s="10"/>
+      <c r="B51" s="10"/>
+      <c r="C51" s="10"/>
+      <c r="D51" s="10"/>
+      <c r="E51" s="10"/>
+      <c r="F51" s="10"/>
       <c r="G51" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="H51" s="11"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="13" t="s">
+      <c r="H51" s="10"/>
+    </row>
+    <row r="52" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A52" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B52" s="23"/>
-      <c r="C52" s="13" t="s">
+      <c r="B52" s="22"/>
+      <c r="C52" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D52" s="13" t="s">
+      <c r="D52" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E52" s="13" t="s">
+      <c r="E52" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F52" s="13" t="s">
+      <c r="F52" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G52" s="13" t="s">
+      <c r="G52" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="H52" s="13" t="s">
+      <c r="H52" s="12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="16"/>
+    <row r="53" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A53" s="15"/>
       <c r="B53" s="4" t="s">
         <v>131</v>
       </c>
       <c r="C53" s="5">
-        <v>0.3333333333333333</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="D53" s="4" t="s">
         <v>132</v>
       </c>
       <c r="E53" s="5">
-        <v>0.2777777777777778</v>
+        <v>0.27777777777777779</v>
       </c>
       <c r="F53" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G53" s="18" t="s">
+      <c r="G53" s="17" t="s">
         <v>48</v>
       </c>
       <c r="H53" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="16"/>
-      <c r="B54" s="17" t="s">
+    <row r="54" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A54" s="15"/>
+      <c r="B54" s="16" t="s">
         <v>133</v>
       </c>
       <c r="C54" s="5">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="D54" s="17" t="s">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="D54" s="16" t="s">
         <v>134</v>
       </c>
       <c r="E54" s="5">
-        <v>0.2847222222222222</v>
+        <v>0.28472222222222221</v>
       </c>
       <c r="F54" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G54" s="18" t="s">
+      <c r="G54" s="17" t="s">
         <v>52</v>
       </c>
       <c r="H54" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="16"/>
+    <row r="55" spans="1:8" ht="27" x14ac:dyDescent="0.95">
+      <c r="A55" s="15"/>
       <c r="B55" s="4" t="s">
         <v>135</v>
       </c>
       <c r="C55" s="5">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="D55" s="24" t="s">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="D55" s="23" t="s">
         <v>136</v>
       </c>
       <c r="E55" s="5">
-        <v>0.2916666666666667</v>
+        <v>0.29166666666666669</v>
       </c>
       <c r="F55" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G55" s="18" t="s">
+      <c r="G55" s="17" t="s">
         <v>56</v>
       </c>
       <c r="H55" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="16"/>
+    <row r="56" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A56" s="15"/>
       <c r="B56" s="4" t="s">
         <v>137</v>
       </c>
       <c r="C56" s="5">
-        <v>0.3333333333333333</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="D56" s="4" t="s">
         <v>138</v>
@@ -2681,100 +2705,100 @@
       <c r="F56" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G56" s="11"/>
+      <c r="G56" s="10"/>
       <c r="H56" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="16"/>
+    <row r="57" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A57" s="15"/>
       <c r="B57" s="4" t="s">
         <v>139</v>
       </c>
       <c r="C57" s="5">
-        <v>0.3333333333333333</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="D57" s="4" t="s">
         <v>140</v>
       </c>
       <c r="E57" s="5">
-        <v>0.3055555555555556</v>
+        <v>0.30555555555555558</v>
       </c>
       <c r="F57" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G57" s="11"/>
+      <c r="G57" s="10"/>
       <c r="H57" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="20"/>
-      <c r="B58" s="20"/>
-      <c r="C58" s="20"/>
-      <c r="D58" s="20"/>
-      <c r="E58" s="20"/>
-      <c r="F58" s="20"/>
-      <c r="G58" s="20"/>
-      <c r="H58" s="20"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="13" t="s">
+    <row r="58" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A58" s="19"/>
+      <c r="B58" s="19"/>
+      <c r="C58" s="19"/>
+      <c r="D58" s="19"/>
+      <c r="E58" s="19"/>
+      <c r="F58" s="19"/>
+      <c r="G58" s="19"/>
+      <c r="H58" s="19"/>
+    </row>
+    <row r="59" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A59" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B59" s="13" t="s">
+      <c r="B59" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C59" s="13" t="s">
+      <c r="C59" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D59" s="13" t="s">
+      <c r="D59" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E59" s="13" t="s">
+      <c r="E59" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F59" s="13" t="s">
+      <c r="F59" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G59" s="13" t="s">
+      <c r="G59" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="H59" s="13" t="s">
+      <c r="H59" s="12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="16"/>
+    <row r="60" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A60" s="15"/>
       <c r="B60" s="4" t="s">
         <v>141</v>
       </c>
       <c r="C60" s="5">
-        <v>0.3333333333333333</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="D60" s="4" t="s">
         <v>142</v>
       </c>
       <c r="E60" s="5">
-        <v>0.2916666666666667</v>
+        <v>0.29166666666666669</v>
       </c>
       <c r="F60" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G60" s="18" t="s">
+      <c r="G60" s="17" t="s">
         <v>66</v>
       </c>
       <c r="H60" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="11"/>
-      <c r="B61" s="25" t="s">
+    <row r="61" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A61" s="10"/>
+      <c r="B61" s="24" t="s">
         <v>143</v>
       </c>
       <c r="C61" s="5">
-        <v>0.3333333333333333</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="D61" s="4" t="s">
         <v>144</v>
@@ -2785,104 +2809,104 @@
       <c r="F61" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G61" s="18" t="s">
+      <c r="G61" s="17" t="s">
         <v>69</v>
       </c>
       <c r="H61" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="11"/>
-      <c r="B62" s="25" t="s">
+    <row r="62" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A62" s="10"/>
+      <c r="B62" s="24" t="s">
         <v>145</v>
       </c>
       <c r="C62" s="5">
-        <v>0.3333333333333333</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="D62" s="4" t="s">
         <v>51</v>
       </c>
       <c r="E62" s="5">
-        <v>0.3090277777777778</v>
+        <v>0.30902777777777779</v>
       </c>
       <c r="F62" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G62" s="18" t="s">
+      <c r="G62" s="17" t="s">
         <v>73</v>
       </c>
       <c r="H62" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="16"/>
+    <row r="63" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A63" s="15"/>
       <c r="B63" s="4" t="s">
         <v>146</v>
       </c>
       <c r="C63" s="5">
-        <v>0.3333333333333333</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="D63" s="4" t="s">
         <v>147</v>
       </c>
       <c r="E63" s="5">
-        <v>0.3159722222222222</v>
+        <v>0.31597222222222221</v>
       </c>
       <c r="F63" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G63" s="11"/>
+      <c r="G63" s="10"/>
       <c r="H63" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="11"/>
-      <c r="B64" s="11"/>
-      <c r="C64" s="11"/>
-      <c r="D64" s="11"/>
-      <c r="E64" s="11"/>
-      <c r="F64" s="11"/>
-      <c r="G64" s="11"/>
-      <c r="H64" s="11"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="13" t="s">
+    <row r="64" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A64" s="10"/>
+      <c r="B64" s="10"/>
+      <c r="C64" s="10"/>
+      <c r="D64" s="10"/>
+      <c r="E64" s="10"/>
+      <c r="F64" s="10"/>
+      <c r="G64" s="10"/>
+      <c r="H64" s="10"/>
+    </row>
+    <row r="65" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A65" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B65" s="13" t="s">
+      <c r="B65" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C65" s="13" t="s">
+      <c r="C65" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D65" s="13" t="s">
+      <c r="D65" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E65" s="13" t="s">
+      <c r="E65" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F65" s="13" t="s">
+      <c r="F65" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G65" s="13" t="s">
+      <c r="G65" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="H65" s="13" t="s">
+      <c r="H65" s="12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="19" t="s">
+    <row r="66" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="A66" s="18" t="s">
         <v>148</v>
       </c>
       <c r="B66" s="4" t="s">
         <v>149</v>
       </c>
       <c r="C66" s="5">
-        <v>0.3333333333333333</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="D66" s="4" t="s">
         <v>150</v>
@@ -2900,7 +2924,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="67">
+    <row r="67" spans="1:8" ht="15" x14ac:dyDescent="0.25">
       <c r="A67" s="4" t="s">
         <v>151</v>
       </c>
@@ -2908,13 +2932,13 @@
         <v>152</v>
       </c>
       <c r="C67" s="5">
-        <v>0.3333333333333333</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="D67" s="4" t="s">
         <v>153</v>
       </c>
       <c r="E67" s="5">
-        <v>0.3055555555555556</v>
+        <v>0.30555555555555558</v>
       </c>
       <c r="F67" s="4" t="s">
         <v>13</v>
@@ -2926,55 +2950,55 @@
         <v>15</v>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="11"/>
-      <c r="B68" s="11"/>
-      <c r="C68" s="26"/>
-      <c r="D68" s="11"/>
-      <c r="E68" s="26"/>
-      <c r="F68" s="11"/>
-      <c r="G68" s="11"/>
-      <c r="H68" s="11"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="13" t="s">
+    <row r="68" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A68" s="10"/>
+      <c r="B68" s="10"/>
+      <c r="C68" s="25"/>
+      <c r="D68" s="10"/>
+      <c r="E68" s="25"/>
+      <c r="F68" s="10"/>
+      <c r="G68" s="10"/>
+      <c r="H68" s="10"/>
+    </row>
+    <row r="69" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A69" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B69" s="13" t="s">
+      <c r="B69" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C69" s="13" t="s">
+      <c r="C69" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D69" s="13" t="s">
+      <c r="D69" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E69" s="13" t="s">
+      <c r="E69" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F69" s="13" t="s">
+      <c r="F69" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G69" s="13" t="s">
+      <c r="G69" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="H69" s="13" t="s">
+      <c r="H69" s="12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="16"/>
+    <row r="70" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="A70" s="15"/>
       <c r="B70" s="4" t="s">
         <v>154</v>
       </c>
       <c r="C70" s="5">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="D70" s="17" t="s">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="D70" s="16" t="s">
         <v>155</v>
       </c>
       <c r="E70" s="5">
-        <v>0.2777777777777778</v>
+        <v>0.27777777777777779</v>
       </c>
       <c r="F70" s="4" t="s">
         <v>13</v>
@@ -2986,7 +3010,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="71">
+    <row r="71" spans="1:8" ht="15" x14ac:dyDescent="0.25">
       <c r="A71" s="4" t="s">
         <v>156</v>
       </c>
@@ -2994,13 +3018,13 @@
         <v>157</v>
       </c>
       <c r="C71" s="5">
-        <v>0.3333333333333333</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="D71" s="4" t="s">
         <v>158</v>
       </c>
       <c r="E71" s="5">
-        <v>0.2847222222222222</v>
+        <v>0.28472222222222221</v>
       </c>
       <c r="F71" s="4" t="s">
         <v>13</v>
@@ -3012,13 +3036,13 @@
         <v>15</v>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="16"/>
+    <row r="72" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="A72" s="15"/>
       <c r="B72" s="4" t="s">
         <v>159</v>
       </c>
       <c r="C72" s="5">
-        <v>0.3333333333333333</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="D72" s="4" t="s">
         <v>160</v>
@@ -3036,7 +3060,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="73">
+    <row r="73" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A73" s="4" t="s">
         <v>161</v>
       </c>
@@ -3044,7 +3068,7 @@
         <v>26</v>
       </c>
       <c r="C73" s="5">
-        <v>0.3333333333333333</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="D73" s="4" t="s">
         <v>162</v>
@@ -3055,12 +3079,12 @@
       <c r="F73" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G73" s="11"/>
+      <c r="G73" s="10"/>
       <c r="H73" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="74">
+    <row r="74" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A74" s="4" t="s">
         <v>163</v>
       </c>
@@ -3068,59 +3092,59 @@
         <v>164</v>
       </c>
       <c r="C74" s="5">
-        <v>0.3333333333333333</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="D74" s="4" t="s">
         <v>165</v>
       </c>
       <c r="E74" s="5">
-        <v>0.3090277777777778</v>
+        <v>0.30902777777777779</v>
       </c>
       <c r="F74" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G74" s="27"/>
-      <c r="H74" s="21" t="s">
+      <c r="G74" s="26"/>
+      <c r="H74" s="20" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="11"/>
-      <c r="B75" s="11"/>
-      <c r="C75" s="11"/>
-      <c r="D75" s="11"/>
-      <c r="E75" s="11"/>
-      <c r="F75" s="11"/>
-      <c r="G75" s="11"/>
-      <c r="H75" s="11"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="13" t="s">
+    <row r="75" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A75" s="10"/>
+      <c r="B75" s="10"/>
+      <c r="C75" s="10"/>
+      <c r="D75" s="10"/>
+      <c r="E75" s="10"/>
+      <c r="F75" s="10"/>
+      <c r="G75" s="10"/>
+      <c r="H75" s="10"/>
+    </row>
+    <row r="76" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A76" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B76" s="13" t="s">
+      <c r="B76" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C76" s="13" t="s">
+      <c r="C76" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D76" s="13" t="s">
+      <c r="D76" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E76" s="13" t="s">
+      <c r="E76" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F76" s="13" t="s">
+      <c r="F76" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G76" s="13" t="s">
+      <c r="G76" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="H76" s="13" t="s">
+      <c r="H76" s="12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="77">
+    <row r="77" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A77" s="4" t="s">
         <v>166</v>
       </c>
@@ -3128,7 +3152,7 @@
         <v>167</v>
       </c>
       <c r="C77" s="5">
-        <v>0.4791666666666667</v>
+        <v>0.47916666666666669</v>
       </c>
       <c r="D77" s="4" t="s">
         <v>168</v>
@@ -3136,37 +3160,37 @@
       <c r="E77" s="5">
         <v>0.4375</v>
       </c>
-      <c r="F77" s="11"/>
-      <c r="G77" s="18" t="s">
+      <c r="F77" s="10"/>
+      <c r="G77" s="17" t="s">
         <v>48</v>
       </c>
       <c r="H77" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="16"/>
+    <row r="78" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A78" s="15"/>
       <c r="B78" s="4" t="s">
         <v>169</v>
       </c>
       <c r="C78" s="5">
-        <v>0.4791666666666667</v>
+        <v>0.47916666666666669</v>
       </c>
       <c r="D78" s="4" t="s">
         <v>170</v>
       </c>
       <c r="E78" s="5">
-        <v>0.4444444444444444</v>
-      </c>
-      <c r="F78" s="11"/>
-      <c r="G78" s="18" t="s">
+        <v>0.44444444444444442</v>
+      </c>
+      <c r="F78" s="10"/>
+      <c r="G78" s="17" t="s">
         <v>52</v>
       </c>
       <c r="H78" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="79">
+    <row r="79" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A79" s="4" t="s">
         <v>171</v>
       </c>
@@ -3174,7 +3198,7 @@
         <v>172</v>
       </c>
       <c r="C79" s="5">
-        <v>0.4791666666666667</v>
+        <v>0.47916666666666669</v>
       </c>
       <c r="D79" s="4" t="s">
         <v>173</v>
@@ -3182,21 +3206,21 @@
       <c r="E79" s="5">
         <v>0.4513888888888889</v>
       </c>
-      <c r="F79" s="11"/>
-      <c r="G79" s="18" t="s">
+      <c r="F79" s="10"/>
+      <c r="G79" s="17" t="s">
         <v>56</v>
       </c>
       <c r="H79" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" s="16"/>
+    <row r="80" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A80" s="15"/>
       <c r="B80" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C80" s="5">
-        <v>0.4791666666666667</v>
+        <v>0.47916666666666669</v>
       </c>
       <c r="D80" s="4" t="s">
         <v>175</v>
@@ -3204,13 +3228,13 @@
       <c r="E80" s="5">
         <v>0.4548611111111111</v>
       </c>
-      <c r="F80" s="11"/>
-      <c r="G80" s="11"/>
+      <c r="F80" s="10"/>
+      <c r="G80" s="10"/>
       <c r="H80" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="81">
+    <row r="81" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A81" s="4" t="s">
         <v>176</v>
       </c>
@@ -3218,57 +3242,57 @@
         <v>177</v>
       </c>
       <c r="C81" s="5">
-        <v>0.4791666666666667</v>
+        <v>0.47916666666666669</v>
       </c>
       <c r="D81" s="4" t="s">
         <v>178</v>
       </c>
       <c r="E81" s="5">
-        <v>0.4583333333333333</v>
-      </c>
-      <c r="F81" s="11"/>
-      <c r="G81" s="11"/>
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="F81" s="10"/>
+      <c r="G81" s="10"/>
       <c r="H81" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" s="11"/>
-      <c r="B82" s="11"/>
-      <c r="C82" s="11"/>
-      <c r="D82" s="11"/>
-      <c r="E82" s="11"/>
-      <c r="F82" s="11"/>
-      <c r="G82" s="11"/>
-      <c r="H82" s="11"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="13" t="s">
+    <row r="82" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A82" s="10"/>
+      <c r="B82" s="10"/>
+      <c r="C82" s="10"/>
+      <c r="D82" s="10"/>
+      <c r="E82" s="10"/>
+      <c r="F82" s="10"/>
+      <c r="G82" s="10"/>
+      <c r="H82" s="10"/>
+    </row>
+    <row r="83" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A83" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B83" s="13" t="s">
+      <c r="B83" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C83" s="13" t="s">
+      <c r="C83" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D83" s="13" t="s">
+      <c r="D83" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E83" s="13" t="s">
+      <c r="E83" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F83" s="13" t="s">
+      <c r="F83" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G83" s="13" t="s">
+      <c r="G83" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="H83" s="13" t="s">
+      <c r="H83" s="12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="84">
+    <row r="84" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A84" s="4" t="s">
         <v>179</v>
       </c>
@@ -3276,23 +3300,23 @@
         <v>180</v>
       </c>
       <c r="C84" s="5">
-        <v>0.4791666666666667</v>
+        <v>0.47916666666666669</v>
       </c>
       <c r="D84" s="4" t="s">
         <v>181</v>
       </c>
       <c r="E84" s="5">
-        <v>0.4479166666666667</v>
-      </c>
-      <c r="F84" s="11"/>
-      <c r="G84" s="18" t="s">
+        <v>0.44791666666666669</v>
+      </c>
+      <c r="F84" s="10"/>
+      <c r="G84" s="17" t="s">
         <v>66</v>
       </c>
       <c r="H84" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="85">
+    <row r="85" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A85" s="4" t="s">
         <v>182</v>
       </c>
@@ -3300,61 +3324,61 @@
         <v>183</v>
       </c>
       <c r="C85" s="5">
-        <v>0.4791666666666667</v>
+        <v>0.47916666666666669</v>
       </c>
       <c r="D85" s="4" t="s">
         <v>18</v>
       </c>
       <c r="E85" s="5">
-        <v>0.4583333333333333</v>
-      </c>
-      <c r="F85" s="11"/>
-      <c r="G85" s="18" t="s">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="F85" s="10"/>
+      <c r="G85" s="17" t="s">
         <v>69</v>
       </c>
       <c r="H85" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" s="11"/>
-      <c r="B86" s="11"/>
-      <c r="C86" s="11"/>
-      <c r="D86" s="11"/>
-      <c r="E86" s="11"/>
-      <c r="F86" s="11"/>
-      <c r="G86" s="18" t="s">
+    <row r="86" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A86" s="10"/>
+      <c r="B86" s="10"/>
+      <c r="C86" s="10"/>
+      <c r="D86" s="10"/>
+      <c r="E86" s="10"/>
+      <c r="F86" s="10"/>
+      <c r="G86" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="H86" s="11"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="13" t="s">
+      <c r="H86" s="10"/>
+    </row>
+    <row r="87" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A87" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B87" s="13" t="s">
+      <c r="B87" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C87" s="13" t="s">
+      <c r="C87" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D87" s="13" t="s">
+      <c r="D87" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E87" s="13" t="s">
+      <c r="E87" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F87" s="13" t="s">
+      <c r="F87" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G87" s="13" t="s">
+      <c r="G87" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="H87" s="13" t="s">
+      <c r="H87" s="12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="88">
+    <row r="88" spans="1:8" ht="15" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
         <v>184</v>
       </c>
@@ -3362,23 +3386,23 @@
         <v>185</v>
       </c>
       <c r="C88" s="5">
-        <v>0.4791666666666667</v>
+        <v>0.47916666666666669</v>
       </c>
       <c r="D88" s="4" t="s">
         <v>186</v>
       </c>
       <c r="E88" s="5">
-        <v>0.4305555555555556</v>
-      </c>
-      <c r="F88" s="11"/>
+        <v>0.43055555555555558</v>
+      </c>
+      <c r="F88" s="10"/>
       <c r="G88" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="H88" s="21" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="89">
+      <c r="H88" s="20" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" ht="15" x14ac:dyDescent="0.25">
       <c r="A89" s="4" t="s">
         <v>187</v>
       </c>
@@ -3386,15 +3410,15 @@
         <v>188</v>
       </c>
       <c r="C89" s="5">
-        <v>0.4791666666666667</v>
+        <v>0.47916666666666669</v>
       </c>
       <c r="D89" s="4" t="s">
         <v>189</v>
       </c>
       <c r="E89" s="5">
-        <v>0.4479166666666667</v>
-      </c>
-      <c r="F89" s="11"/>
+        <v>0.44791666666666669</v>
+      </c>
+      <c r="F89" s="10"/>
       <c r="G89" s="6" t="s">
         <v>19</v>
       </c>
@@ -3402,15 +3426,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" s="15" t="s">
+    <row r="90" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="A90" s="14" t="s">
         <v>190</v>
       </c>
       <c r="B90" s="4" t="s">
         <v>191</v>
       </c>
       <c r="C90" s="5">
-        <v>0.4791666666666667</v>
+        <v>0.47916666666666669</v>
       </c>
       <c r="D90" s="4" t="s">
         <v>40</v>
@@ -3418,15 +3442,15 @@
       <c r="E90" s="5">
         <v>0.4548611111111111</v>
       </c>
-      <c r="F90" s="11"/>
+      <c r="F90" s="10"/>
       <c r="G90" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="H90" s="21" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="91">
+      <c r="H90" s="20" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A91" s="4" t="s">
         <v>192</v>
       </c>
@@ -3434,21 +3458,21 @@
         <v>193</v>
       </c>
       <c r="C91" s="5">
-        <v>0.4791666666666667</v>
+        <v>0.47916666666666669</v>
       </c>
       <c r="D91" s="4" t="s">
         <v>194</v>
       </c>
       <c r="E91" s="5">
-        <v>0.4583333333333333</v>
-      </c>
-      <c r="F91" s="11"/>
-      <c r="G91" s="27"/>
-      <c r="H91" s="21" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="92">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="F91" s="10"/>
+      <c r="G91" s="26"/>
+      <c r="H91" s="20" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A92" s="4" t="s">
         <v>195</v>
       </c>
@@ -3456,145 +3480,145 @@
         <v>196</v>
       </c>
       <c r="C92" s="5">
-        <v>0.4791666666666667</v>
+        <v>0.47916666666666669</v>
       </c>
       <c r="D92" s="4" t="s">
         <v>197</v>
       </c>
       <c r="E92" s="5">
-        <v>0.4618055555555556</v>
-      </c>
-      <c r="F92" s="11"/>
-      <c r="G92" s="11"/>
+        <v>0.46180555555555558</v>
+      </c>
+      <c r="F92" s="10"/>
+      <c r="G92" s="10"/>
       <c r="H92" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" s="11"/>
-      <c r="B93" s="11"/>
-      <c r="C93" s="26"/>
-      <c r="D93" s="11"/>
-      <c r="E93" s="26"/>
-      <c r="F93" s="11"/>
-      <c r="G93" s="11"/>
-      <c r="H93" s="11"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="13" t="s">
+    <row r="93" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A93" s="10"/>
+      <c r="B93" s="10"/>
+      <c r="C93" s="25"/>
+      <c r="D93" s="10"/>
+      <c r="E93" s="25"/>
+      <c r="F93" s="10"/>
+      <c r="G93" s="10"/>
+      <c r="H93" s="10"/>
+    </row>
+    <row r="94" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A94" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B94" s="13" t="s">
+      <c r="B94" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C94" s="13" t="s">
+      <c r="C94" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D94" s="13" t="s">
+      <c r="D94" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E94" s="13" t="s">
+      <c r="E94" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F94" s="13" t="s">
+      <c r="F94" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G94" s="13" t="s">
+      <c r="G94" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="H94" s="13" t="s">
+      <c r="H94" s="12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" s="16"/>
+    <row r="95" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="A95" s="15"/>
       <c r="B95" s="4" t="s">
         <v>198</v>
       </c>
       <c r="C95" s="5">
-        <v>0.4583333333333333</v>
+        <v>0.45833333333333331</v>
       </c>
       <c r="D95" s="4" t="s">
         <v>198</v>
       </c>
       <c r="E95" s="5">
-        <v>0.4340277777777778</v>
-      </c>
-      <c r="F95" s="11"/>
+        <v>0.43402777777777779</v>
+      </c>
+      <c r="F95" s="10"/>
       <c r="G95" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="H95" s="21" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="19" t="s">
+      <c r="H95" s="20" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="A96" s="18" t="s">
         <v>199</v>
       </c>
       <c r="B96" s="4" t="s">
         <v>58</v>
       </c>
       <c r="C96" s="5">
-        <v>0.4583333333333333</v>
+        <v>0.45833333333333331</v>
       </c>
       <c r="D96" s="4" t="s">
         <v>59</v>
       </c>
       <c r="E96" s="5">
-        <v>0.4409722222222222</v>
-      </c>
-      <c r="F96" s="11"/>
+        <v>0.44097222222222221</v>
+      </c>
+      <c r="F96" s="10"/>
       <c r="G96" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="H96" s="21" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="20"/>
-      <c r="B97" s="20"/>
-      <c r="C97" s="20"/>
-      <c r="D97" s="20"/>
-      <c r="E97" s="20"/>
-      <c r="F97" s="20"/>
-      <c r="G97" s="28"/>
-      <c r="H97" s="20"/>
-    </row>
-    <row r="98">
-      <c r="A98" s="13" t="s">
+      <c r="H96" s="20" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A97" s="19"/>
+      <c r="B97" s="19"/>
+      <c r="C97" s="19"/>
+      <c r="D97" s="19"/>
+      <c r="E97" s="19"/>
+      <c r="F97" s="19"/>
+      <c r="G97" s="27"/>
+      <c r="H97" s="19"/>
+    </row>
+    <row r="98" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A98" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B98" s="13" t="s">
+      <c r="B98" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C98" s="13" t="s">
+      <c r="C98" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D98" s="13" t="s">
+      <c r="D98" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E98" s="13" t="s">
+      <c r="E98" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F98" s="13" t="s">
+      <c r="F98" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G98" s="13" t="s">
+      <c r="G98" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="H98" s="13" t="s">
+      <c r="H98" s="12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="99">
-      <c r="A99" s="16"/>
+    <row r="99" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="A99" s="15"/>
       <c r="B99" s="4" t="s">
         <v>200</v>
       </c>
       <c r="C99" s="5">
-        <v>0.4166666666666667</v>
+        <v>0.41666666666666669</v>
       </c>
       <c r="D99" s="4" t="s">
         <v>200</v>
@@ -3602,7 +3626,7 @@
       <c r="E99" s="5">
         <v>0.3888888888888889</v>
       </c>
-      <c r="F99" s="11"/>
+      <c r="F99" s="10"/>
       <c r="G99" s="6" t="s">
         <v>75</v>
       </c>
@@ -3610,13 +3634,13 @@
         <v>15</v>
       </c>
     </row>
-    <row r="100">
-      <c r="A100" s="16"/>
+    <row r="100" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="A100" s="15"/>
       <c r="B100" s="4" t="s">
         <v>200</v>
       </c>
       <c r="C100" s="5">
-        <v>0.4166666666666667</v>
+        <v>0.41666666666666669</v>
       </c>
       <c r="D100" s="4" t="s">
         <v>200</v>
@@ -3624,7 +3648,7 @@
       <c r="E100" s="5">
         <v>0.3888888888888889</v>
       </c>
-      <c r="F100" s="11"/>
+      <c r="F100" s="10"/>
       <c r="G100" s="6" t="s">
         <v>79</v>
       </c>
@@ -3632,13 +3656,13 @@
         <v>15</v>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" s="16"/>
+    <row r="101" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="A101" s="15"/>
       <c r="B101" s="4" t="s">
         <v>200</v>
       </c>
       <c r="C101" s="5">
-        <v>0.4166666666666667</v>
+        <v>0.41666666666666669</v>
       </c>
       <c r="D101" s="4" t="s">
         <v>200</v>
@@ -3646,7 +3670,7 @@
       <c r="E101" s="5">
         <v>0.3888888888888889</v>
       </c>
-      <c r="F101" s="11"/>
+      <c r="F101" s="10"/>
       <c r="G101" s="6" t="s">
         <v>83</v>
       </c>
@@ -3654,13 +3678,13 @@
         <v>24</v>
       </c>
     </row>
-    <row r="102">
-      <c r="A102" s="16"/>
+    <row r="102" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A102" s="15"/>
       <c r="B102" s="4" t="s">
         <v>200</v>
       </c>
       <c r="C102" s="5">
-        <v>0.4166666666666667</v>
+        <v>0.41666666666666669</v>
       </c>
       <c r="D102" s="4" t="s">
         <v>200</v>
@@ -3668,19 +3692,19 @@
       <c r="E102" s="5">
         <v>0.3888888888888889</v>
       </c>
-      <c r="F102" s="11"/>
-      <c r="G102" s="11"/>
+      <c r="F102" s="10"/>
+      <c r="G102" s="10"/>
       <c r="H102" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="103">
-      <c r="A103" s="11"/>
+    <row r="103" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A103" s="10"/>
       <c r="B103" s="4" t="s">
         <v>200</v>
       </c>
       <c r="C103" s="5">
-        <v>0.4166666666666667</v>
+        <v>0.41666666666666669</v>
       </c>
       <c r="D103" s="4" t="s">
         <v>200</v>
@@ -3688,16 +3712,16 @@
       <c r="E103" s="5">
         <v>0.3888888888888889</v>
       </c>
-      <c r="F103" s="11"/>
-      <c r="G103" s="11"/>
+      <c r="F103" s="10"/>
+      <c r="G103" s="10"/>
       <c r="H103" s="4" t="s">
         <v>24</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>